<commit_message>
code update and commit
</commit_message>
<xml_diff>
--- a/Test Data/OutputData.xlsx
+++ b/Test Data/OutputData.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4143" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4441" uniqueCount="194">
   <si>
     <t>DetailsDBData</t>
   </si>
@@ -601,6 +601,9 @@
   </si>
   <si>
     <t>62703</t>
+  </si>
+  <si>
+    <t>ISP</t>
   </si>
 </sst>
 </file>
@@ -1615,7 +1618,7 @@
     </row>
     <row r="8">
       <c r="C8" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D8" t="s">
         <v>189</v>

</xml_diff>